<commit_message>
feat(update): enhance employee update assertions, navigation stability, and auto-venv execution
</commit_message>
<xml_diff>
--- a/update/emp_mgmt/test_data/Swarajya-Update-Employee-test-cases.xlsx
+++ b/update/emp_mgmt/test_data/Swarajya-Update-Employee-test-cases.xlsx
@@ -1497,9 +1497,9 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1549,9 +1549,9 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1601,9 +1601,9 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1704,9 +1704,9 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1807,9 +1807,9 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1959,9 +1959,9 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="J12" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -2010,9 +2010,9 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="J13" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -2061,9 +2061,9 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="J14" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(update): restructure employee update architecture to match vendor management standards
</commit_message>
<xml_diff>
--- a/update/emp_mgmt/test_data/Swarajya-Update-Employee-test-cases.xlsx
+++ b/update/emp_mgmt/test_data/Swarajya-Update-Employee-test-cases.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Update_Positive_Flows" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Update_Negative_Flows" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update_Positive_Flows" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update_Negative_Flows" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -577,7 +577,11 @@
           <t>The employee profile is updated successfully with the new mandatory details and a confirmation message is displayed.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="n"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>AUT_TC_POS_UPD_001</t>
+        </is>
+      </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Automated</t>
@@ -1435,7 +1439,11 @@
           <t>Update submission fails and a validation error is displayed indicating the mandatory field cannot be blank.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="n"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>AUT_TC_NEG_UPD_001</t>
+        </is>
+      </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Automated</t>

</xml_diff>